<commit_message>
Make corrections from validation of harmo output
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{46D68B9B-100B-4F03-AA1C-0C879900D0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4775CBE1-C9C6-422B-A919-D82E763BEECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="788">
   <si>
     <t>index</t>
   </si>
@@ -2605,9 +2605,6 @@
     <t>I think the variable b11mensy6 is about Women's Health, and other variables I see don't seem appropriate for the DS variable.</t>
   </si>
   <si>
-    <t>The study-specific variable asks about types of health problems since last interview/2016.</t>
-  </si>
-  <si>
     <t>The study-specific variable asks about types of health problems (Raised cholesterol) since last interview/2016.</t>
   </si>
   <si>
@@ -2669,20 +2666,6 @@
   <si>
     <t>Type of cancer has had since last interview/2016: Breast cancer ; 
 Health problems since last interview/2016: Cancer or leukaemia</t>
-  </si>
-  <si>
-    <t>case_when(
-b11ccty06 == 1 ~ 1L ; 
-b11ccty06 == 0 ~ 0L ;
-b11khlpb05 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-b11ccty04 == 1 ~ 1L ; 
-b11ccty04 == 0 ~ 0L ;
-b11khlpb05 == 0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
   </si>
   <si>
     <t>b11ccty04 ;
@@ -2726,19 +2709,6 @@
 up to A-levels or diploma (typically age 18 years) and degree or higher." 
 Diploma =&gt; Grade 11/12
 Do not need to use NVQ.</t>
-  </si>
-  <si>
-    <t>recode(
-0=0;
-1=0;
-2=0;
-3=1;
-4=1;
-5=1;
-7=1;
-8=1;
--1=NA;
-ELSE=NA)</t>
   </si>
   <si>
     <t>Recoding as in Wave 1:
@@ -2879,13 +2849,6 @@
 ELSE=NA)</t>
   </si>
   <si>
-    <t>recode(
-3=1;
-4=2;
--9:-1=NA;
-ELSE=NA)</t>
-  </si>
-  <si>
     <t>Study-specific responses only available for daily smokers, not for occasional smokers.</t>
   </si>
   <si>
@@ -2990,33 +2953,6 @@
 Health problems since last interview/2016: Heart problems</t>
   </si>
   <si>
-    <t>The study-specific variable asks about types of heart problems since last interview/2016.</t>
-  </si>
-  <si>
-    <t>case_when(
-b11hrtp2 == 1 ~ 1L ; 
-b11hrtp2 == 0 ~ 0L ; 
-b11khlpb08 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-b11hrtp1 == 1 ~ 1L ; 
-b11hrtp1 == 0 ~ 0L ; 
-b11khlpb08 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>case_when(
-b11hrtp3 == 1 ~ 1L ; 
-b11hrtp3 == 0 ~ 0L ; 
-b11khlpb08 == 0 ~ 0L ;
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>recode(0 = 0 ; 1 = 1 ; -9:-1 = NA ; ELSE = NA)</t>
-  </si>
-  <si>
     <t>The study variable has Yes/No so can code No.</t>
   </si>
   <si>
@@ -3036,10 +2972,6 @@
   </si>
   <si>
     <t>recode(0 = NA ; 1 = 1 ; ELSE = NA)</t>
-  </si>
-  <si>
-    <t>The study-specific variables ask about types of health since last interview/2016. 
-Arthritis coded as 1=Yes. Could not assign 0=No.</t>
   </si>
   <si>
     <t>recode(
@@ -3190,6 +3122,85 @@
   </si>
   <si>
     <t>Modified to use same algorithm as baseline.</t>
+  </si>
+  <si>
+    <t>Kept as presumed no here because categories are mentioned/not mentioned. In Baseline, they are Yes/No.</t>
+  </si>
+  <si>
+    <t>case_when(
+b11hrtp2 == 1 ~ 1L ; 
+b11hrtp2 == 0 ~ 2L ; 
+b11khlpb08 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+b11hrtp1 == 1 ~ 1L ; 
+b11hrtp1 == 0 ~ 2L ; 
+b11khlpb08 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+b11hrtp3 == 1 ~ 1L ; 
+b11hrtp3 == 0 ~ 2L ; 
+b11khlpb08 == 0 ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>recode(0 = 2 ; 1 = 1 ; -9:-1 = NA ; ELSE = NA)</t>
+  </si>
+  <si>
+    <t>case_when(
+b11ccty06 == 1 ~ 1L ; 
+b11ccty06 == 0 ~ 2L ;
+b11khlpb05 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+b11ccty04 == 1 ~ 1L ; 
+b11ccty04 == 0 ~ 2L ;
+b11khlpb05 == 0 ~ 2L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of health problems since last interview/2016.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of heart problems since last interview/2016.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>The study-specific variables ask about types of health since last interview/2016. 
+Arthritis coded as 1=Yes. Could not assign Presumed no.</t>
+  </si>
+  <si>
+    <t>The study-specific variable asks about types of cancer since last interview/2016.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.</t>
+  </si>
+  <si>
+    <t>recode(
+3=1;
+4=2;
+1:2 = NA ;
+-9:-1=NA;
+ELSE=NA)</t>
+  </si>
+  <si>
+    <t>recode(
+0=0;
+1=0;
+2=0;
+3=1;
+4=1;
+5=1;
+6 =1;
+7=1;
+8=1;
+-1=NA;
+ELSE=NA)</t>
   </si>
 </sst>
 </file>
@@ -3758,7 +3769,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -3971,7 +3982,7 @@
         <v>50</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>781</v>
+        <v>770</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -4047,7 +4058,7 @@
         <v>68</v>
       </c>
       <c r="V6" s="12" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>41</v>
@@ -4174,7 +4185,7 @@
         <v>93</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
     <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
@@ -4218,7 +4229,7 @@
         <v>102</v>
       </c>
       <c r="V9" s="12" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>41</v>
@@ -4230,22 +4241,22 @@
         <v>79</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>103</v>
       </c>
       <c r="AB9" s="24" t="s">
+        <v>704</v>
+      </c>
+      <c r="AC9" s="12" t="s">
         <v>707</v>
       </c>
-      <c r="AC9" s="12" t="s">
-        <v>711</v>
-      </c>
       <c r="AD9" s="24" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="10" spans="1:33" ht="165" x14ac:dyDescent="0.25">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" ht="180" x14ac:dyDescent="0.25">
       <c r="A10" s="16">
         <v>9</v>
       </c>
@@ -4295,13 +4306,13 @@
         <v>79</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>709</v>
+        <v>787</v>
       </c>
       <c r="AC10" s="12" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="AD10" s="24" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
     </row>
     <row r="11" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -4348,7 +4359,7 @@
         <v>117</v>
       </c>
       <c r="V11" s="12" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>41</v>
@@ -4360,10 +4371,10 @@
         <v>79</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="AC11" s="2" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="12" spans="1:33" ht="195" x14ac:dyDescent="0.25">
@@ -4413,7 +4424,7 @@
         <v>124</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>41</v>
@@ -4451,10 +4462,10 @@
         <v>129</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="O13" s="23"/>
       <c r="P13" s="23" t="s">
@@ -4466,10 +4477,10 @@
         <v>131</v>
       </c>
       <c r="T13" s="25" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="U13" s="18" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>41</v>
@@ -4481,13 +4492,13 @@
         <v>92</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="AA13" s="18" t="s">
         <v>132</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
     </row>
     <row r="14" spans="1:33" ht="409.5" x14ac:dyDescent="0.25">
@@ -4522,7 +4533,7 @@
         <v>138</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>41</v>
@@ -4534,13 +4545,13 @@
         <v>79</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="AA14" s="18" t="s">
         <v>139</v>
       </c>
       <c r="AC14" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -4584,7 +4595,7 @@
         <v>117</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>41</v>
@@ -4640,7 +4651,7 @@
         <v>155</v>
       </c>
       <c r="V16" s="12" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>41</v>
@@ -4693,7 +4704,7 @@
         <v>165</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>41</v>
@@ -4761,7 +4772,7 @@
         <v>179</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>41</v>
@@ -4779,7 +4790,7 @@
         <v>181</v>
       </c>
       <c r="AC18" s="18" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -4888,7 +4899,7 @@
         <v>190</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="W20" s="16" t="s">
         <v>41</v>
@@ -5961,10 +5972,10 @@
         <v>297</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>779</v>
+        <v>768</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>778</v>
+        <v>767</v>
       </c>
       <c r="O45" s="23" t="s">
         <v>298</v>
@@ -5974,10 +5985,10 @@
       <c r="R45" s="23"/>
       <c r="S45" s="23"/>
       <c r="T45" s="2" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="V45" s="12" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="W45" s="23" t="s">
         <v>41</v>
@@ -5989,7 +6000,7 @@
         <v>92</v>
       </c>
       <c r="Z45" s="22" t="s">
-        <v>780</v>
+        <v>769</v>
       </c>
       <c r="AA45" s="18" t="s">
         <v>299</v>
@@ -5998,7 +6009,7 @@
         <v>300</v>
       </c>
       <c r="AC45" s="22" t="s">
-        <v>777</v>
+        <v>766</v>
       </c>
       <c r="AD45" s="19" t="s">
         <v>675</v>
@@ -6034,7 +6045,7 @@
       </c>
       <c r="O46" s="23"/>
       <c r="P46" s="23" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="Q46" s="23"/>
       <c r="R46" s="23"/>
@@ -6043,7 +6054,7 @@
         <v>672</v>
       </c>
       <c r="V46" s="11" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="W46" s="13" t="s">
         <v>41</v>
@@ -6055,10 +6066,10 @@
         <v>79</v>
       </c>
       <c r="Z46" s="2" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="AD46" s="22" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6108,7 +6119,7 @@
         <v>314</v>
       </c>
       <c r="V47" s="12" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="W47" s="16" t="s">
         <v>41</v>
@@ -6120,7 +6131,7 @@
         <v>79</v>
       </c>
       <c r="Z47" s="2" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6164,7 +6175,7 @@
         <v>314</v>
       </c>
       <c r="V48" s="12" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="W48" s="16" t="s">
         <v>41</v>
@@ -6176,7 +6187,7 @@
         <v>79</v>
       </c>
       <c r="Z48" s="2" t="s">
-        <v>737</v>
+        <v>786</v>
       </c>
     </row>
     <row r="49" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -6217,7 +6228,7 @@
         <v>324</v>
       </c>
       <c r="V49" s="12" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="W49" s="16" t="s">
         <v>41</v>
@@ -6229,13 +6240,13 @@
         <v>92</v>
       </c>
       <c r="Z49" s="2" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="AA49" s="18" t="s">
         <v>325</v>
       </c>
       <c r="AC49" s="2" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
     </row>
     <row r="50" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -6385,7 +6396,7 @@
         <v>345</v>
       </c>
       <c r="V52" s="12" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="W52" s="16" t="s">
         <v>213</v>
@@ -6406,10 +6417,10 @@
         <v>347</v>
       </c>
       <c r="AC52" s="2" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="AD52" s="24" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
     </row>
     <row r="53" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -6450,7 +6461,7 @@
         <v>355</v>
       </c>
       <c r="V53" s="12" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="W53" s="16" t="s">
         <v>41</v>
@@ -6462,13 +6473,13 @@
         <v>92</v>
       </c>
       <c r="Z53" s="2" t="s">
-        <v>784</v>
+        <v>773</v>
       </c>
       <c r="AA53" s="18" t="s">
         <v>356</v>
       </c>
       <c r="AC53" s="2" t="s">
-        <v>785</v>
+        <v>774</v>
       </c>
     </row>
     <row r="54" spans="1:30" ht="150" x14ac:dyDescent="0.25">
@@ -6509,7 +6520,7 @@
         <v>355</v>
       </c>
       <c r="V54" s="12" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>41</v>
@@ -6559,7 +6570,7 @@
         <v>355</v>
       </c>
       <c r="V55" s="12" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="W55" s="16" t="s">
         <v>41</v>
@@ -6703,7 +6714,7 @@
         <v>379</v>
       </c>
       <c r="AC58" s="2" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.25">
@@ -6829,7 +6840,7 @@
         <v>395</v>
       </c>
       <c r="V61" s="12" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>41</v>
@@ -6882,7 +6893,7 @@
         <v>404</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>41</v>
@@ -6938,7 +6949,7 @@
         <v>412</v>
       </c>
       <c r="V63" s="12" t="s">
-        <v>749</v>
+        <v>744</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>41</v>
@@ -6997,7 +7008,7 @@
         <v>423</v>
       </c>
       <c r="V64" s="11" t="s">
-        <v>750</v>
+        <v>745</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>41</v>
@@ -7041,7 +7052,7 @@
         <v>107</v>
       </c>
       <c r="M65" s="18" t="s">
-        <v>783</v>
+        <v>772</v>
       </c>
       <c r="N65" s="18" t="s">
         <v>429</v>
@@ -7056,7 +7067,7 @@
         <v>412</v>
       </c>
       <c r="V65" s="2" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="W65" s="16" t="s">
         <v>41</v>
@@ -7259,10 +7270,10 @@
         <v>467</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="O69" s="16" t="s">
         <v>468</v>
@@ -7274,7 +7285,7 @@
         <v>470</v>
       </c>
       <c r="V69" s="12" t="s">
-        <v>679</v>
+        <v>782</v>
       </c>
       <c r="W69" s="16" t="s">
         <v>41</v>
@@ -7286,7 +7297,7 @@
         <v>92</v>
       </c>
       <c r="Z69" s="2" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="AA69" s="18" t="s">
         <v>471</v>
@@ -7295,7 +7306,7 @@
         <v>472</v>
       </c>
       <c r="AC69" s="12" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
     </row>
     <row r="70" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7327,10 +7338,10 @@
         <v>467</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="O70" s="23" t="s">
         <v>468</v>
@@ -7340,10 +7351,10 @@
       <c r="R70" s="23"/>
       <c r="S70" s="23"/>
       <c r="T70" s="2" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="V70" s="12" t="s">
-        <v>763</v>
+        <v>783</v>
       </c>
       <c r="W70" s="23" t="s">
         <v>41</v>
@@ -7355,13 +7366,13 @@
         <v>92</v>
       </c>
       <c r="Z70" s="2" t="s">
-        <v>764</v>
+        <v>776</v>
       </c>
       <c r="AB70" s="18" t="s">
         <v>673</v>
       </c>
       <c r="AC70" s="2" t="s">
-        <v>769</v>
+        <v>759</v>
       </c>
     </row>
     <row r="71" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7393,10 +7404,10 @@
         <v>467</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="O71" s="23" t="s">
         <v>482</v>
@@ -7406,10 +7417,10 @@
       <c r="R71" s="23"/>
       <c r="S71" s="23"/>
       <c r="T71" s="2" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="V71" s="12" t="s">
-        <v>763</v>
+        <v>783</v>
       </c>
       <c r="W71" s="23" t="s">
         <v>41</v>
@@ -7421,10 +7432,10 @@
         <v>92</v>
       </c>
       <c r="Z71" s="2" t="s">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="AC71" s="2" t="s">
-        <v>769</v>
+        <v>759</v>
       </c>
     </row>
     <row r="72" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7456,10 +7467,10 @@
         <v>467</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="O72" s="23" t="s">
         <v>482</v>
@@ -7469,10 +7480,10 @@
       <c r="R72" s="23"/>
       <c r="S72" s="23"/>
       <c r="T72" s="2" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="V72" s="12" t="s">
-        <v>763</v>
+        <v>783</v>
       </c>
       <c r="W72" s="23" t="s">
         <v>41</v>
@@ -7484,10 +7495,10 @@
         <v>92</v>
       </c>
       <c r="Z72" s="2" t="s">
-        <v>766</v>
+        <v>778</v>
       </c>
       <c r="AC72" s="2" t="s">
-        <v>769</v>
+        <v>759</v>
       </c>
     </row>
     <row r="73" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7534,7 +7545,7 @@
         <v>470</v>
       </c>
       <c r="V73" s="12" t="s">
-        <v>679</v>
+        <v>782</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>41</v>
@@ -7546,13 +7557,13 @@
         <v>79</v>
       </c>
       <c r="Z73" s="2" t="s">
-        <v>767</v>
+        <v>779</v>
       </c>
       <c r="AA73" s="18" t="s">
         <v>494</v>
       </c>
       <c r="AC73" s="2" t="s">
-        <v>768</v>
+        <v>758</v>
       </c>
     </row>
     <row r="74" spans="1:30" x14ac:dyDescent="0.25">
@@ -7646,7 +7657,7 @@
         <v>213</v>
       </c>
       <c r="AC75" s="18" t="s">
-        <v>770</v>
+        <v>760</v>
       </c>
     </row>
     <row r="76" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7695,6 +7706,9 @@
       <c r="T76" s="21" t="s">
         <v>470</v>
       </c>
+      <c r="V76" s="12" t="s">
+        <v>782</v>
+      </c>
       <c r="W76" s="16" t="s">
         <v>41</v>
       </c>
@@ -7705,13 +7719,13 @@
         <v>79</v>
       </c>
       <c r="Z76" s="2" t="s">
-        <v>767</v>
+        <v>779</v>
       </c>
       <c r="AA76" s="18" t="s">
         <v>511</v>
       </c>
       <c r="AC76" s="2" t="s">
-        <v>768</v>
+        <v>758</v>
       </c>
     </row>
     <row r="77" spans="1:30" x14ac:dyDescent="0.25">
@@ -7758,7 +7772,7 @@
         <v>213</v>
       </c>
       <c r="AC77" s="18" t="s">
-        <v>771</v>
+        <v>761</v>
       </c>
     </row>
     <row r="78" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7790,17 +7804,17 @@
         <v>467</v>
       </c>
       <c r="M78" s="2" t="s">
-        <v>773</v>
+        <v>763</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>772</v>
+        <v>762</v>
       </c>
       <c r="O78" s="16" t="s">
         <v>521</v>
       </c>
       <c r="T78" s="2"/>
       <c r="V78" s="12" t="s">
-        <v>775</v>
+        <v>784</v>
       </c>
       <c r="W78" s="23" t="s">
         <v>41</v>
@@ -7812,7 +7826,7 @@
         <v>79</v>
       </c>
       <c r="Z78" s="2" t="s">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="AB78" s="11" t="s">
         <v>472</v>
@@ -7874,13 +7888,16 @@
         <v>79</v>
       </c>
       <c r="Z79" s="2" t="s">
-        <v>776</v>
+        <v>765</v>
       </c>
       <c r="AA79" s="18" t="s">
         <v>529</v>
       </c>
       <c r="AB79" s="11" t="s">
         <v>472</v>
+      </c>
+      <c r="AC79" s="2" t="s">
+        <v>775</v>
       </c>
     </row>
     <row r="80" spans="1:30" x14ac:dyDescent="0.25">
@@ -7970,6 +7987,9 @@
       <c r="T81" s="21" t="s">
         <v>470</v>
       </c>
+      <c r="V81" s="12" t="s">
+        <v>782</v>
+      </c>
       <c r="W81" s="16" t="s">
         <v>41</v>
       </c>
@@ -7980,7 +8000,7 @@
         <v>79</v>
       </c>
       <c r="Z81" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="AA81" s="18" t="s">
         <v>541</v>
@@ -8021,28 +8041,28 @@
         <v>548</v>
       </c>
       <c r="W82" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X82" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y82" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z82" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA82" s="18" t="s">
         <v>549</v>
       </c>
       <c r="AB82" s="12" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="AC82" s="2" t="s">
         <v>674</v>
       </c>
       <c r="AD82" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="83" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8071,10 +8091,10 @@
         <v>467</v>
       </c>
       <c r="M83" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="N83" s="2" t="s">
         <v>697</v>
-      </c>
-      <c r="N83" s="2" t="s">
-        <v>698</v>
       </c>
       <c r="P83" s="16" t="s">
         <v>548</v>
@@ -8082,6 +8102,9 @@
       <c r="T83" s="21" t="s">
         <v>553</v>
       </c>
+      <c r="V83" s="12" t="s">
+        <v>785</v>
+      </c>
       <c r="W83" s="16" t="s">
         <v>41</v>
       </c>
@@ -8092,13 +8115,13 @@
         <v>92</v>
       </c>
       <c r="Z83" s="2" t="s">
-        <v>699</v>
+        <v>780</v>
       </c>
       <c r="AA83" s="18" t="s">
         <v>554</v>
       </c>
       <c r="AD83" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="84" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8139,25 +8162,25 @@
         <v>553</v>
       </c>
       <c r="W84" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X84" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y84" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z84" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA84" s="18" t="s">
         <v>559</v>
       </c>
       <c r="AB84" s="12" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AD84" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="85" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8198,25 +8221,25 @@
         <v>553</v>
       </c>
       <c r="W85" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X85" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y85" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z85" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA85" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB85" s="12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="AD85" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="86" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8257,25 +8280,25 @@
         <v>553</v>
       </c>
       <c r="W86" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X86" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y86" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z86" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA86" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB86" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="AD86" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="87" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8316,25 +8339,25 @@
         <v>553</v>
       </c>
       <c r="W87" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X87" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y87" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z87" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA87" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB87" s="12" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="AD87" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="88" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8375,25 +8398,25 @@
         <v>553</v>
       </c>
       <c r="W88" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X88" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y88" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z88" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA88" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB88" s="12" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="AD88" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="89" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8434,25 +8457,25 @@
         <v>553</v>
       </c>
       <c r="W89" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X89" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y89" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z89" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA89" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB89" s="12" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="AD89" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8493,25 +8516,25 @@
         <v>553</v>
       </c>
       <c r="W90" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X90" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y90" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z90" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA90" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB90" s="12" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="AD90" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="91" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8552,25 +8575,25 @@
         <v>553</v>
       </c>
       <c r="W91" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X91" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y91" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z91" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA91" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB91" s="12" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="AD91" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="92" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8599,10 +8622,10 @@
         <v>467</v>
       </c>
       <c r="M92" s="2" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="P92" s="16" t="s">
         <v>548</v>
@@ -8610,6 +8633,9 @@
       <c r="T92" s="21" t="s">
         <v>553</v>
       </c>
+      <c r="V92" s="12" t="s">
+        <v>785</v>
+      </c>
       <c r="W92" s="16" t="s">
         <v>41</v>
       </c>
@@ -8620,13 +8646,13 @@
         <v>92</v>
       </c>
       <c r="Z92" s="2" t="s">
-        <v>700</v>
+        <v>781</v>
       </c>
       <c r="AA92" s="18" t="s">
         <v>554</v>
       </c>
       <c r="AD92" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="93" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8667,25 +8693,25 @@
         <v>553</v>
       </c>
       <c r="W93" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X93" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y93" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Z93" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA93" s="18" t="s">
         <v>564</v>
       </c>
       <c r="AB93" s="12" t="s">
+        <v>682</v>
+      </c>
+      <c r="AD93" s="2" t="s">
         <v>683</v>
-      </c>
-      <c r="AD93" s="2" t="s">
-        <v>684</v>
       </c>
     </row>
     <row r="94" spans="1:30" x14ac:dyDescent="0.25">
@@ -9016,7 +9042,7 @@
         <v>470</v>
       </c>
       <c r="V101" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="W101" s="16" t="s">
         <v>41</v>
@@ -9034,7 +9060,7 @@
         <v>623</v>
       </c>
       <c r="AC101" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="102" spans="1:29" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix alcohol quantity algorithm
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4775CBE1-C9C6-422B-A919-D82E763BEECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777DDE27-79CC-4308-BDF5-E84AA1E17250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="790">
   <si>
     <t>index</t>
   </si>
@@ -2716,13 +2716,6 @@
 Coding for study category 6? (not coded)</t>
   </si>
   <si>
-    <t>Recoding as in age Wave 1:
-Agree with GCSE A-C as upper secondary.
-Seems like 7=degree level would usually be ISCED 6, but 'foundation degree' would be ISCED. Added harmo comment about coding.
-Coding for study category 6? (not coded).
-Also a variable BD10ANVQ, but everyone with info for BD10ANVQ has BD10HACHQ. -&gt; Many people have NVQ = 0.</t>
-  </si>
-  <si>
     <t>Study-specific categories 'Unemployed and seeking work (5)' and 'Permanent sickness/disability (9)'were coded as DataSchema category 'Unemployed'.
 Study-specific categories 'In full-time education (6)', 'On a government scheme for employment training (7)', 'Temporarily sick/disabled (8)', 'Looking after home or family (10)', 'Wholly retired (11)', ' Something else (12)' were considered unknown/NA.</t>
   </si>
@@ -3008,23 +3001,6 @@
 b11winstg;
 b11winsmg;
 b11alcopp</t>
-  </si>
-  <si>
-    <t>case_when(
-  b11drink08 == 1 ~ 0L,
-  ELSE ~ rowSums(mutate(., 
-    b11beern_units = case_when(b11beern &lt; 0 ~ NA_real_ , TRUE ~ b11beern * 2) ,
-    b11beers_units = case_when(b11beers &lt; 0 ~ NA_real_ , TRUE ~ b11beers * 3) ,
-    b11spiris_units = case_when(b11spiris &lt; 0 ~ NA_real_ , TRUE ~ b11spiris * 1) ,
-    b11sherry_units = case_when(b11sherry &lt; 0 ~ NA_real_ , TRUE ~ b11sherry * 1) ,
-    b11winebt_units = case_when(b11winebt &lt; 0 ~ NA_real_ , TRUE ~ b11winebt * 1.5) ,
-    b11winlag_units = case_when(b11winlag &lt; 0 ~ NA_real_ , TRUE ~ b11winlag * 3),
-    b11winstg_units = case_when(b11winstg &lt; 0 ~ NA_real_ , TRUE ~ b11winstg * 2.1),
-    b11winsmg_units = case_when(b11winsmg &lt; 0 ~ NA_real_ , TRUE ~ b11winsmg * 1.5),
-    b11alcopp_units = case_when(b11alcopp &lt; 0 ~ NA_real_ , TRUE ~ b11alcopp * 1.5)
-  ) %&gt;%
-    select(ends_with("_units")), na.rm = TRUE)
-)</t>
   </si>
   <si>
     <t>Only one population.</t>
@@ -3201,6 +3177,38 @@
 8=1;
 -1=NA;
 ELSE=NA)</t>
+  </si>
+  <si>
+    <t>case_when(
+  b11drink08 == 1 ~ 0L,
+  ELSE ~ rowSums(mutate(., 
+    b11beern_units = case_when(b11beern &lt; 0 ~ NA_real_ , TRUE ~ b11beern * 2) ,
+    b11beers_units = case_when(b11beers &lt; 0 ~ NA_real_ , TRUE ~ b11beers * 3) ,
+    b11spiris_units = case_when(b11spiris &lt; 0 ~ NA_real_ , TRUE ~ b11spiris * 1) ,
+    b11sherry_units = case_when(b11sherry &lt; 0 ~ NA_real_ , TRUE ~ b11sherry * 1) ,
+    b11winebt_units = case_when(b11winebt &lt; 0 ~ NA_real_ , TRUE ~ b11winebt * 1.5) ,
+    b11winlag_units = case_when(b11winlag &lt; 0 ~ NA_real_ , TRUE ~ b11winlag * 3),
+    b11winstg_units = case_when(b11winstg &lt; 0 ~ NA_real_ , TRUE ~ b11winstg * 2.1),
+    b11winsmg_units = case_when(b11winsmg &lt; 0 ~ NA_real_ , TRUE ~ b11winsmg * 1.5),
+    b11alcopp_units = case_when(b11alcopp &lt; 0 ~ NA_real_ , TRUE ~ b11alcopp * 1.5)
+  ) %&gt;%
+    select(ends_with("_units")), na.rm = TRUE) * 8
+)</t>
+  </si>
+  <si>
+    <t>(Derived) Highest Academic Qualification obtained up to age 51</t>
+  </si>
+  <si>
+    <t>bd11hachq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The input variable appeared to be incorrect (almost all 0). Check that this is the correct one to use.
+Recoding as in age Wave 1:
+Agree with GCSE A-C as upper secondary.
+Seems like 7=degree level would usually be ISCED 6, but 'foundation degree' would be ISCED. Added harmo comment about coding.
+Coding for study category 6? (not coded).
+Also a variable BD10ANVQ, but everyone with info for BD10ANVQ has BD10HACHQ. -&gt; Many people have NVQ = 0.
+</t>
   </si>
 </sst>
 </file>
@@ -3769,7 +3777,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -3982,7 +3990,7 @@
         <v>50</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -4188,7 +4196,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" ht="210" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>8</v>
       </c>
@@ -4216,11 +4224,11 @@
       <c r="L9" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="M9" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="N9" s="18" t="s">
-        <v>101</v>
+      <c r="M9" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>787</v>
       </c>
       <c r="S9" s="16" t="s">
         <v>58</v>
@@ -4249,8 +4257,8 @@
       <c r="AB9" s="24" t="s">
         <v>704</v>
       </c>
-      <c r="AC9" s="12" t="s">
-        <v>707</v>
+      <c r="AC9" s="11" t="s">
+        <v>789</v>
       </c>
       <c r="AD9" s="24" t="s">
         <v>705</v>
@@ -4306,7 +4314,7 @@
         <v>79</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="AC10" s="12" t="s">
         <v>706</v>
@@ -4359,7 +4367,7 @@
         <v>117</v>
       </c>
       <c r="V11" s="12" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>41</v>
@@ -4371,10 +4379,10 @@
         <v>79</v>
       </c>
       <c r="Z11" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="AC11" s="2" t="s">
         <v>709</v>
-      </c>
-      <c r="AC11" s="2" t="s">
-        <v>710</v>
       </c>
     </row>
     <row r="12" spans="1:33" ht="195" x14ac:dyDescent="0.25">
@@ -4424,7 +4432,7 @@
         <v>124</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>41</v>
@@ -4462,10 +4470,10 @@
         <v>129</v>
       </c>
       <c r="M13" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>712</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>713</v>
       </c>
       <c r="O13" s="23"/>
       <c r="P13" s="23" t="s">
@@ -4477,10 +4485,10 @@
         <v>131</v>
       </c>
       <c r="T13" s="25" t="s">
+        <v>713</v>
+      </c>
+      <c r="U13" s="18" t="s">
         <v>714</v>
-      </c>
-      <c r="U13" s="18" t="s">
-        <v>715</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>41</v>
@@ -4492,13 +4500,13 @@
         <v>92</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="AA13" s="18" t="s">
         <v>132</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="14" spans="1:33" ht="409.5" x14ac:dyDescent="0.25">
@@ -4533,7 +4541,7 @@
         <v>138</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>41</v>
@@ -4545,7 +4553,7 @@
         <v>79</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="AA14" s="18" t="s">
         <v>139</v>
@@ -4595,7 +4603,7 @@
         <v>117</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>41</v>
@@ -4651,7 +4659,7 @@
         <v>155</v>
       </c>
       <c r="V16" s="12" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>41</v>
@@ -4704,7 +4712,7 @@
         <v>165</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>41</v>
@@ -4772,7 +4780,7 @@
         <v>179</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>41</v>
@@ -4790,7 +4798,7 @@
         <v>181</v>
       </c>
       <c r="AC18" s="18" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -4899,7 +4907,7 @@
         <v>190</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="W20" s="16" t="s">
         <v>41</v>
@@ -5972,10 +5980,10 @@
         <v>297</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="O45" s="23" t="s">
         <v>298</v>
@@ -5985,10 +5993,10 @@
       <c r="R45" s="23"/>
       <c r="S45" s="23"/>
       <c r="T45" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="V45" s="12" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="W45" s="23" t="s">
         <v>41</v>
@@ -5999,8 +6007,8 @@
       <c r="Y45" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="Z45" s="22" t="s">
-        <v>769</v>
+      <c r="Z45" s="2" t="s">
+        <v>786</v>
       </c>
       <c r="AA45" s="18" t="s">
         <v>299</v>
@@ -6008,8 +6016,8 @@
       <c r="AB45" s="24" t="s">
         <v>300</v>
       </c>
-      <c r="AC45" s="22" t="s">
-        <v>766</v>
+      <c r="AC45" s="2" t="s">
+        <v>765</v>
       </c>
       <c r="AD45" s="19" t="s">
         <v>675</v>
@@ -6045,7 +6053,7 @@
       </c>
       <c r="O46" s="23"/>
       <c r="P46" s="23" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="Q46" s="23"/>
       <c r="R46" s="23"/>
@@ -6053,8 +6061,8 @@
       <c r="T46" s="2" t="s">
         <v>672</v>
       </c>
-      <c r="V46" s="11" t="s">
-        <v>729</v>
+      <c r="V46" s="12" t="s">
+        <v>728</v>
       </c>
       <c r="W46" s="13" t="s">
         <v>41</v>
@@ -6066,10 +6074,10 @@
         <v>79</v>
       </c>
       <c r="Z46" s="2" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="AD46" s="22" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6119,7 +6127,7 @@
         <v>314</v>
       </c>
       <c r="V47" s="12" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="W47" s="16" t="s">
         <v>41</v>
@@ -6131,7 +6139,7 @@
         <v>79</v>
       </c>
       <c r="Z47" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6175,7 +6183,7 @@
         <v>314</v>
       </c>
       <c r="V48" s="12" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="W48" s="16" t="s">
         <v>41</v>
@@ -6187,7 +6195,7 @@
         <v>79</v>
       </c>
       <c r="Z48" s="2" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="49" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -6228,7 +6236,7 @@
         <v>324</v>
       </c>
       <c r="V49" s="12" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="W49" s="16" t="s">
         <v>41</v>
@@ -6240,13 +6248,13 @@
         <v>92</v>
       </c>
       <c r="Z49" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="AA49" s="18" t="s">
         <v>325</v>
       </c>
       <c r="AC49" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="50" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -6396,7 +6404,7 @@
         <v>345</v>
       </c>
       <c r="V52" s="12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="W52" s="16" t="s">
         <v>213</v>
@@ -6417,10 +6425,10 @@
         <v>347</v>
       </c>
       <c r="AC52" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="AD52" s="24" t="s">
         <v>736</v>
-      </c>
-      <c r="AD52" s="24" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="53" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -6461,7 +6469,7 @@
         <v>355</v>
       </c>
       <c r="V53" s="12" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="W53" s="16" t="s">
         <v>41</v>
@@ -6473,13 +6481,13 @@
         <v>92</v>
       </c>
       <c r="Z53" s="2" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="AA53" s="18" t="s">
         <v>356</v>
       </c>
       <c r="AC53" s="2" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="54" spans="1:30" ht="150" x14ac:dyDescent="0.25">
@@ -6520,7 +6528,7 @@
         <v>355</v>
       </c>
       <c r="V54" s="12" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>41</v>
@@ -6570,7 +6578,7 @@
         <v>355</v>
       </c>
       <c r="V55" s="12" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="W55" s="16" t="s">
         <v>41</v>
@@ -6714,7 +6722,7 @@
         <v>379</v>
       </c>
       <c r="AC58" s="2" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.25">
@@ -6840,7 +6848,7 @@
         <v>395</v>
       </c>
       <c r="V61" s="12" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>41</v>
@@ -6893,7 +6901,7 @@
         <v>404</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>41</v>
@@ -6949,7 +6957,7 @@
         <v>412</v>
       </c>
       <c r="V63" s="12" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>41</v>
@@ -7008,7 +7016,7 @@
         <v>423</v>
       </c>
       <c r="V64" s="11" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>41</v>
@@ -7052,7 +7060,7 @@
         <v>107</v>
       </c>
       <c r="M65" s="18" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="N65" s="18" t="s">
         <v>429</v>
@@ -7067,7 +7075,7 @@
         <v>412</v>
       </c>
       <c r="V65" s="2" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="W65" s="16" t="s">
         <v>41</v>
@@ -7270,10 +7278,10 @@
         <v>467</v>
       </c>
       <c r="M69" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="N69" s="2" t="s">
         <v>748</v>
-      </c>
-      <c r="N69" s="2" t="s">
-        <v>749</v>
       </c>
       <c r="O69" s="16" t="s">
         <v>468</v>
@@ -7285,7 +7293,7 @@
         <v>470</v>
       </c>
       <c r="V69" s="12" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="W69" s="16" t="s">
         <v>41</v>
@@ -7297,7 +7305,7 @@
         <v>92</v>
       </c>
       <c r="Z69" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="AA69" s="18" t="s">
         <v>471</v>
@@ -7306,7 +7314,7 @@
         <v>472</v>
       </c>
       <c r="AC69" s="12" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="70" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7338,10 +7346,10 @@
         <v>467</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="O70" s="23" t="s">
         <v>468</v>
@@ -7351,10 +7359,10 @@
       <c r="R70" s="23"/>
       <c r="S70" s="23"/>
       <c r="T70" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="V70" s="12" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="W70" s="23" t="s">
         <v>41</v>
@@ -7366,13 +7374,13 @@
         <v>92</v>
       </c>
       <c r="Z70" s="2" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="AB70" s="18" t="s">
         <v>673</v>
       </c>
       <c r="AC70" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="71" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7404,10 +7412,10 @@
         <v>467</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="O71" s="23" t="s">
         <v>482</v>
@@ -7417,10 +7425,10 @@
       <c r="R71" s="23"/>
       <c r="S71" s="23"/>
       <c r="T71" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="V71" s="12" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="W71" s="23" t="s">
         <v>41</v>
@@ -7432,10 +7440,10 @@
         <v>92</v>
       </c>
       <c r="Z71" s="2" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="AC71" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="72" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7467,10 +7475,10 @@
         <v>467</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="O72" s="23" t="s">
         <v>482</v>
@@ -7480,10 +7488,10 @@
       <c r="R72" s="23"/>
       <c r="S72" s="23"/>
       <c r="T72" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="V72" s="12" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="W72" s="23" t="s">
         <v>41</v>
@@ -7495,10 +7503,10 @@
         <v>92</v>
       </c>
       <c r="Z72" s="2" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="AC72" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="73" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7545,7 +7553,7 @@
         <v>470</v>
       </c>
       <c r="V73" s="12" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>41</v>
@@ -7557,13 +7565,13 @@
         <v>79</v>
       </c>
       <c r="Z73" s="2" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="AA73" s="18" t="s">
         <v>494</v>
       </c>
       <c r="AC73" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="74" spans="1:30" x14ac:dyDescent="0.25">
@@ -7657,7 +7665,7 @@
         <v>213</v>
       </c>
       <c r="AC75" s="18" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="76" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7707,7 +7715,7 @@
         <v>470</v>
       </c>
       <c r="V76" s="12" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="W76" s="16" t="s">
         <v>41</v>
@@ -7719,13 +7727,13 @@
         <v>79</v>
       </c>
       <c r="Z76" s="2" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="AA76" s="18" t="s">
         <v>511</v>
       </c>
       <c r="AC76" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="77" spans="1:30" x14ac:dyDescent="0.25">
@@ -7772,7 +7780,7 @@
         <v>213</v>
       </c>
       <c r="AC77" s="18" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="78" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7804,17 +7812,17 @@
         <v>467</v>
       </c>
       <c r="M78" s="2" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="O78" s="16" t="s">
         <v>521</v>
       </c>
       <c r="T78" s="2"/>
       <c r="V78" s="12" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="W78" s="23" t="s">
         <v>41</v>
@@ -7826,7 +7834,7 @@
         <v>79</v>
       </c>
       <c r="Z78" s="2" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="AB78" s="11" t="s">
         <v>472</v>
@@ -7888,7 +7896,7 @@
         <v>79</v>
       </c>
       <c r="Z79" s="2" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="AA79" s="18" t="s">
         <v>529</v>
@@ -7897,7 +7905,7 @@
         <v>472</v>
       </c>
       <c r="AC79" s="2" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
     </row>
     <row r="80" spans="1:30" x14ac:dyDescent="0.25">
@@ -7988,7 +7996,7 @@
         <v>470</v>
       </c>
       <c r="V81" s="12" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="W81" s="16" t="s">
         <v>41</v>
@@ -8103,7 +8111,7 @@
         <v>553</v>
       </c>
       <c r="V83" s="12" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="W83" s="16" t="s">
         <v>41</v>
@@ -8115,7 +8123,7 @@
         <v>92</v>
       </c>
       <c r="Z83" s="2" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="AA83" s="18" t="s">
         <v>554</v>
@@ -8634,7 +8642,7 @@
         <v>553</v>
       </c>
       <c r="V92" s="12" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="W92" s="16" t="s">
         <v>41</v>
@@ -8646,7 +8654,7 @@
         <v>92</v>
       </c>
       <c r="Z92" s="2" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="AA92" s="18" t="s">
         <v>554</v>

</xml_diff>

<commit_message>
Change input variable b11ccty50 to BLANK
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777DDE27-79CC-4308-BDF5-E84AA1E17250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9832A0F6-2A33-4765-9E49-BED7F11A0A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="789">
   <si>
     <t>index</t>
   </si>
@@ -2167,9 +2167,6 @@
     <t>If the study-specific variable has Yes/No responses, the harmonized values can be Yes/No. 
 If the study-specific variable is conditional on a parent variable with Yes/No responses (e.g., Have you ever had any cancer? Yes/No) or there is a response option for "None of the above" for a list including this cancer, the harmonized values can be Yes/No. 
 If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
-  </si>
-  <si>
-    <t>b11ccty50</t>
   </si>
   <si>
     <t>Type of cancer has had since last interview/2016: Bladder</t>
@@ -3777,7 +3774,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -3990,7 +3987,7 @@
         <v>50</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -4066,7 +4063,7 @@
         <v>68</v>
       </c>
       <c r="V6" s="12" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>41</v>
@@ -4184,16 +4181,16 @@
         <v>42</v>
       </c>
       <c r="Y8" s="13" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="Z8" s="13" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="AA8" s="18" t="s">
         <v>93</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="9" spans="1:33" ht="210" x14ac:dyDescent="0.25">
@@ -4225,10 +4222,10 @@
         <v>99</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="S9" s="16" t="s">
         <v>58</v>
@@ -4237,7 +4234,7 @@
         <v>102</v>
       </c>
       <c r="V9" s="12" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>41</v>
@@ -4249,19 +4246,19 @@
         <v>79</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>103</v>
       </c>
       <c r="AB9" s="24" t="s">
+        <v>703</v>
+      </c>
+      <c r="AC9" s="11" t="s">
+        <v>788</v>
+      </c>
+      <c r="AD9" s="24" t="s">
         <v>704</v>
-      </c>
-      <c r="AC9" s="11" t="s">
-        <v>789</v>
-      </c>
-      <c r="AD9" s="24" t="s">
-        <v>705</v>
       </c>
     </row>
     <row r="10" spans="1:33" ht="180" x14ac:dyDescent="0.25">
@@ -4314,13 +4311,13 @@
         <v>79</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="AC10" s="12" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="AD10" s="24" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="11" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -4367,7 +4364,7 @@
         <v>117</v>
       </c>
       <c r="V11" s="12" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>41</v>
@@ -4379,10 +4376,10 @@
         <v>79</v>
       </c>
       <c r="Z11" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="AC11" s="2" t="s">
         <v>708</v>
-      </c>
-      <c r="AC11" s="2" t="s">
-        <v>709</v>
       </c>
     </row>
     <row r="12" spans="1:33" ht="195" x14ac:dyDescent="0.25">
@@ -4432,7 +4429,7 @@
         <v>124</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>41</v>
@@ -4470,10 +4467,10 @@
         <v>129</v>
       </c>
       <c r="M13" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>711</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>712</v>
       </c>
       <c r="O13" s="23"/>
       <c r="P13" s="23" t="s">
@@ -4485,10 +4482,10 @@
         <v>131</v>
       </c>
       <c r="T13" s="25" t="s">
+        <v>712</v>
+      </c>
+      <c r="U13" s="18" t="s">
         <v>713</v>
-      </c>
-      <c r="U13" s="18" t="s">
-        <v>714</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>41</v>
@@ -4500,13 +4497,13 @@
         <v>92</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="AA13" s="18" t="s">
         <v>132</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="14" spans="1:33" ht="409.5" x14ac:dyDescent="0.25">
@@ -4541,7 +4538,7 @@
         <v>138</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>41</v>
@@ -4553,13 +4550,13 @@
         <v>79</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="AA14" s="18" t="s">
         <v>139</v>
       </c>
       <c r="AC14" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="285" x14ac:dyDescent="0.25">
@@ -4603,7 +4600,7 @@
         <v>117</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>41</v>
@@ -4659,7 +4656,7 @@
         <v>155</v>
       </c>
       <c r="V16" s="12" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>41</v>
@@ -4712,7 +4709,7 @@
         <v>165</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>41</v>
@@ -4780,7 +4777,7 @@
         <v>179</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>41</v>
@@ -4798,7 +4795,7 @@
         <v>181</v>
       </c>
       <c r="AC18" s="18" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -4907,7 +4904,7 @@
         <v>190</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="W20" s="16" t="s">
         <v>41</v>
@@ -5980,10 +5977,10 @@
         <v>297</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="O45" s="23" t="s">
         <v>298</v>
@@ -5993,10 +5990,10 @@
       <c r="R45" s="23"/>
       <c r="S45" s="23"/>
       <c r="T45" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="V45" s="12" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="W45" s="23" t="s">
         <v>41</v>
@@ -6008,7 +6005,7 @@
         <v>92</v>
       </c>
       <c r="Z45" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="AA45" s="18" t="s">
         <v>299</v>
@@ -6017,10 +6014,10 @@
         <v>300</v>
       </c>
       <c r="AC45" s="2" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="AD45" s="19" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="46" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -6046,23 +6043,23 @@
         <v>303</v>
       </c>
       <c r="M46" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="N46" s="2" t="s">
         <v>670</v>
-      </c>
-      <c r="N46" s="2" t="s">
-        <v>671</v>
       </c>
       <c r="O46" s="23"/>
       <c r="P46" s="23" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="Q46" s="23"/>
       <c r="R46" s="23"/>
       <c r="S46" s="23"/>
       <c r="T46" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="V46" s="12" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="W46" s="13" t="s">
         <v>41</v>
@@ -6074,10 +6071,10 @@
         <v>79</v>
       </c>
       <c r="Z46" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AD46" s="22" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6127,7 +6124,7 @@
         <v>314</v>
       </c>
       <c r="V47" s="12" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="W47" s="16" t="s">
         <v>41</v>
@@ -6139,7 +6136,7 @@
         <v>79</v>
       </c>
       <c r="Z47" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="165" x14ac:dyDescent="0.25">
@@ -6183,7 +6180,7 @@
         <v>314</v>
       </c>
       <c r="V48" s="12" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="W48" s="16" t="s">
         <v>41</v>
@@ -6195,7 +6192,7 @@
         <v>79</v>
       </c>
       <c r="Z48" s="2" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="49" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -6236,7 +6233,7 @@
         <v>324</v>
       </c>
       <c r="V49" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="W49" s="16" t="s">
         <v>41</v>
@@ -6248,13 +6245,13 @@
         <v>92</v>
       </c>
       <c r="Z49" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="AA49" s="18" t="s">
         <v>325</v>
       </c>
       <c r="AC49" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="50" spans="1:30" ht="45" x14ac:dyDescent="0.25">
@@ -6404,7 +6401,7 @@
         <v>345</v>
       </c>
       <c r="V52" s="12" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="W52" s="16" t="s">
         <v>213</v>
@@ -6425,10 +6422,10 @@
         <v>347</v>
       </c>
       <c r="AC52" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="AD52" s="24" t="s">
         <v>735</v>
-      </c>
-      <c r="AD52" s="24" t="s">
-        <v>736</v>
       </c>
     </row>
     <row r="53" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
@@ -6469,7 +6466,7 @@
         <v>355</v>
       </c>
       <c r="V53" s="12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="W53" s="16" t="s">
         <v>41</v>
@@ -6481,13 +6478,13 @@
         <v>92</v>
       </c>
       <c r="Z53" s="2" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="AA53" s="18" t="s">
         <v>356</v>
       </c>
       <c r="AC53" s="2" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="54" spans="1:30" ht="150" x14ac:dyDescent="0.25">
@@ -6528,7 +6525,7 @@
         <v>355</v>
       </c>
       <c r="V54" s="12" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>41</v>
@@ -6578,7 +6575,7 @@
         <v>355</v>
       </c>
       <c r="V55" s="12" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="W55" s="16" t="s">
         <v>41</v>
@@ -6722,7 +6719,7 @@
         <v>379</v>
       </c>
       <c r="AC58" s="2" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.25">
@@ -6848,7 +6845,7 @@
         <v>395</v>
       </c>
       <c r="V61" s="12" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>41</v>
@@ -6901,7 +6898,7 @@
         <v>404</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>41</v>
@@ -6957,7 +6954,7 @@
         <v>412</v>
       </c>
       <c r="V63" s="12" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>41</v>
@@ -7016,7 +7013,7 @@
         <v>423</v>
       </c>
       <c r="V64" s="11" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>41</v>
@@ -7060,7 +7057,7 @@
         <v>107</v>
       </c>
       <c r="M65" s="18" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="N65" s="18" t="s">
         <v>429</v>
@@ -7075,7 +7072,7 @@
         <v>412</v>
       </c>
       <c r="V65" s="2" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="W65" s="16" t="s">
         <v>41</v>
@@ -7143,7 +7140,7 @@
         <v>441</v>
       </c>
       <c r="AD66" s="18" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="67" spans="1:30" ht="150" x14ac:dyDescent="0.25">
@@ -7278,10 +7275,10 @@
         <v>467</v>
       </c>
       <c r="M69" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="N69" s="2" t="s">
         <v>747</v>
-      </c>
-      <c r="N69" s="2" t="s">
-        <v>748</v>
       </c>
       <c r="O69" s="16" t="s">
         <v>468</v>
@@ -7293,7 +7290,7 @@
         <v>470</v>
       </c>
       <c r="V69" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W69" s="16" t="s">
         <v>41</v>
@@ -7305,7 +7302,7 @@
         <v>92</v>
       </c>
       <c r="Z69" s="2" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="AA69" s="18" t="s">
         <v>471</v>
@@ -7314,7 +7311,7 @@
         <v>472</v>
       </c>
       <c r="AC69" s="12" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="70" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7346,10 +7343,10 @@
         <v>467</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="O70" s="23" t="s">
         <v>468</v>
@@ -7359,10 +7356,10 @@
       <c r="R70" s="23"/>
       <c r="S70" s="23"/>
       <c r="T70" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="V70" s="12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="W70" s="23" t="s">
         <v>41</v>
@@ -7374,13 +7371,13 @@
         <v>92</v>
       </c>
       <c r="Z70" s="2" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="AB70" s="18" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="AC70" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="71" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7412,10 +7409,10 @@
         <v>467</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="O71" s="23" t="s">
         <v>482</v>
@@ -7425,10 +7422,10 @@
       <c r="R71" s="23"/>
       <c r="S71" s="23"/>
       <c r="T71" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="V71" s="12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="W71" s="23" t="s">
         <v>41</v>
@@ -7440,10 +7437,10 @@
         <v>92</v>
       </c>
       <c r="Z71" s="2" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="AC71" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="72" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -7475,10 +7472,10 @@
         <v>467</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="O72" s="23" t="s">
         <v>482</v>
@@ -7488,10 +7485,10 @@
       <c r="R72" s="23"/>
       <c r="S72" s="23"/>
       <c r="T72" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="V72" s="12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="W72" s="23" t="s">
         <v>41</v>
@@ -7503,10 +7500,10 @@
         <v>92</v>
       </c>
       <c r="Z72" s="2" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="AC72" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="73" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7553,7 +7550,7 @@
         <v>470</v>
       </c>
       <c r="V73" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>41</v>
@@ -7565,13 +7562,13 @@
         <v>79</v>
       </c>
       <c r="Z73" s="2" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AA73" s="18" t="s">
         <v>494</v>
       </c>
       <c r="AC73" s="2" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="74" spans="1:30" x14ac:dyDescent="0.25">
@@ -7665,7 +7662,7 @@
         <v>213</v>
       </c>
       <c r="AC75" s="18" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="76" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -7715,7 +7712,7 @@
         <v>470</v>
       </c>
       <c r="V76" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W76" s="16" t="s">
         <v>41</v>
@@ -7727,13 +7724,13 @@
         <v>79</v>
       </c>
       <c r="Z76" s="2" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AA76" s="18" t="s">
         <v>511</v>
       </c>
       <c r="AC76" s="2" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="77" spans="1:30" x14ac:dyDescent="0.25">
@@ -7780,7 +7777,7 @@
         <v>213</v>
       </c>
       <c r="AC77" s="18" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="78" spans="1:30" ht="90" x14ac:dyDescent="0.25">
@@ -7812,17 +7809,17 @@
         <v>467</v>
       </c>
       <c r="M78" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="O78" s="16" t="s">
         <v>521</v>
       </c>
       <c r="T78" s="2"/>
       <c r="V78" s="12" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="W78" s="23" t="s">
         <v>41</v>
@@ -7834,7 +7831,7 @@
         <v>79</v>
       </c>
       <c r="Z78" s="2" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AB78" s="11" t="s">
         <v>472</v>
@@ -7896,7 +7893,7 @@
         <v>79</v>
       </c>
       <c r="Z79" s="2" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="AA79" s="18" t="s">
         <v>529</v>
@@ -7905,7 +7902,7 @@
         <v>472</v>
       </c>
       <c r="AC79" s="2" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="80" spans="1:30" x14ac:dyDescent="0.25">
@@ -7996,7 +7993,7 @@
         <v>470</v>
       </c>
       <c r="V81" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W81" s="16" t="s">
         <v>41</v>
@@ -8008,7 +8005,7 @@
         <v>79</v>
       </c>
       <c r="Z81" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="AA81" s="18" t="s">
         <v>541</v>
@@ -8040,37 +8037,37 @@
         <v>467</v>
       </c>
       <c r="M82" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N82" s="18" t="s">
         <v>546</v>
       </c>
-      <c r="N82" s="18" t="s">
+      <c r="P82" s="16" t="s">
         <v>547</v>
       </c>
-      <c r="P82" s="16" t="s">
+      <c r="W82" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="X82" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y82" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Z82" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="AA82" s="18" t="s">
         <v>548</v>
       </c>
-      <c r="W82" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="X82" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Y82" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Z82" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="AA82" s="18" t="s">
-        <v>549</v>
-      </c>
       <c r="AB82" s="12" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AC82" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="AD82" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="83" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8081,13 +8078,13 @@
         <v>32</v>
       </c>
       <c r="C83" s="16" t="s">
+        <v>549</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>550</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="E83" s="16" t="s">
         <v>551</v>
-      </c>
-      <c r="E83" s="16" t="s">
-        <v>552</v>
       </c>
       <c r="F83" s="16" t="s">
         <v>58</v>
@@ -8099,19 +8096,19 @@
         <v>467</v>
       </c>
       <c r="M83" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="N83" s="2" t="s">
         <v>696</v>
       </c>
-      <c r="N83" s="2" t="s">
-        <v>697</v>
-      </c>
       <c r="P83" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T83" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="V83" s="12" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="W83" s="16" t="s">
         <v>41</v>
@@ -8123,13 +8120,13 @@
         <v>92</v>
       </c>
       <c r="Z83" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="AA83" s="18" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="AD83" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="84" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8140,13 +8137,13 @@
         <v>32</v>
       </c>
       <c r="C84" s="16" t="s">
+        <v>554</v>
+      </c>
+      <c r="D84" s="16" t="s">
         <v>555</v>
       </c>
-      <c r="D84" s="16" t="s">
+      <c r="E84" s="16" t="s">
         <v>556</v>
-      </c>
-      <c r="E84" s="16" t="s">
-        <v>557</v>
       </c>
       <c r="F84" s="16" t="s">
         <v>58</v>
@@ -8161,34 +8158,34 @@
         <v>48</v>
       </c>
       <c r="N84" s="18" t="s">
+        <v>557</v>
+      </c>
+      <c r="P84" s="16" t="s">
+        <v>547</v>
+      </c>
+      <c r="T84" s="21" t="s">
+        <v>552</v>
+      </c>
+      <c r="W84" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="X84" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y84" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Z84" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="AA84" s="18" t="s">
         <v>558</v>
       </c>
-      <c r="P84" s="16" t="s">
-        <v>548</v>
-      </c>
-      <c r="T84" s="21" t="s">
-        <v>553</v>
-      </c>
-      <c r="W84" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="X84" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Y84" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Z84" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="AA84" s="18" t="s">
-        <v>559</v>
-      </c>
       <c r="AB84" s="12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="AD84" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="85" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8199,13 +8196,13 @@
         <v>32</v>
       </c>
       <c r="C85" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="D85" s="16" t="s">
         <v>560</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="E85" s="16" t="s">
         <v>561</v>
-      </c>
-      <c r="E85" s="16" t="s">
-        <v>562</v>
       </c>
       <c r="F85" s="16" t="s">
         <v>58</v>
@@ -8220,34 +8217,34 @@
         <v>48</v>
       </c>
       <c r="N85" s="18" t="s">
+        <v>562</v>
+      </c>
+      <c r="P85" s="16" t="s">
+        <v>547</v>
+      </c>
+      <c r="T85" s="21" t="s">
+        <v>552</v>
+      </c>
+      <c r="W85" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="X85" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y85" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Z85" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="AA85" s="18" t="s">
         <v>563</v>
       </c>
-      <c r="P85" s="16" t="s">
-        <v>548</v>
-      </c>
-      <c r="T85" s="21" t="s">
-        <v>553</v>
-      </c>
-      <c r="W85" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="X85" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Y85" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Z85" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="AA85" s="18" t="s">
-        <v>564</v>
-      </c>
       <c r="AB85" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="AD85" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="86" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8258,13 +8255,13 @@
         <v>32</v>
       </c>
       <c r="C86" s="16" t="s">
+        <v>564</v>
+      </c>
+      <c r="D86" s="16" t="s">
         <v>565</v>
       </c>
-      <c r="D86" s="16" t="s">
+      <c r="E86" s="16" t="s">
         <v>566</v>
-      </c>
-      <c r="E86" s="16" t="s">
-        <v>567</v>
       </c>
       <c r="F86" s="16" t="s">
         <v>58</v>
@@ -8279,34 +8276,34 @@
         <v>48</v>
       </c>
       <c r="N86" s="18" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="P86" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T86" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W86" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X86" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y86" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z86" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA86" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB86" s="12" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="AD86" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="87" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8317,13 +8314,13 @@
         <v>32</v>
       </c>
       <c r="C87" s="16" t="s">
+        <v>568</v>
+      </c>
+      <c r="D87" s="16" t="s">
         <v>569</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="E87" s="16" t="s">
         <v>570</v>
-      </c>
-      <c r="E87" s="16" t="s">
-        <v>571</v>
       </c>
       <c r="F87" s="16" t="s">
         <v>58</v>
@@ -8338,34 +8335,34 @@
         <v>48</v>
       </c>
       <c r="N87" s="18" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="P87" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T87" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W87" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X87" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y87" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z87" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA87" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB87" s="12" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="AD87" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="88" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8376,13 +8373,13 @@
         <v>32</v>
       </c>
       <c r="C88" s="16" t="s">
+        <v>572</v>
+      </c>
+      <c r="D88" s="16" t="s">
         <v>573</v>
       </c>
-      <c r="D88" s="16" t="s">
+      <c r="E88" s="16" t="s">
         <v>574</v>
-      </c>
-      <c r="E88" s="16" t="s">
-        <v>575</v>
       </c>
       <c r="F88" s="16" t="s">
         <v>58</v>
@@ -8397,34 +8394,34 @@
         <v>48</v>
       </c>
       <c r="N88" s="18" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="P88" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T88" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W88" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X88" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y88" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z88" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA88" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB88" s="12" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="AD88" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="89" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8435,13 +8432,13 @@
         <v>32</v>
       </c>
       <c r="C89" s="16" t="s">
+        <v>576</v>
+      </c>
+      <c r="D89" s="16" t="s">
         <v>577</v>
       </c>
-      <c r="D89" s="16" t="s">
+      <c r="E89" s="16" t="s">
         <v>578</v>
-      </c>
-      <c r="E89" s="16" t="s">
-        <v>579</v>
       </c>
       <c r="F89" s="16" t="s">
         <v>58</v>
@@ -8456,34 +8453,34 @@
         <v>48</v>
       </c>
       <c r="N89" s="18" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="P89" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T89" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W89" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X89" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y89" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z89" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA89" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB89" s="12" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="AD89" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8494,13 +8491,13 @@
         <v>32</v>
       </c>
       <c r="C90" s="16" t="s">
+        <v>580</v>
+      </c>
+      <c r="D90" s="16" t="s">
         <v>581</v>
       </c>
-      <c r="D90" s="16" t="s">
+      <c r="E90" s="16" t="s">
         <v>582</v>
-      </c>
-      <c r="E90" s="16" t="s">
-        <v>583</v>
       </c>
       <c r="F90" s="16" t="s">
         <v>58</v>
@@ -8515,34 +8512,34 @@
         <v>48</v>
       </c>
       <c r="N90" s="18" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="P90" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T90" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W90" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X90" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y90" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z90" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA90" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB90" s="12" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="AD90" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="91" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8553,13 +8550,13 @@
         <v>32</v>
       </c>
       <c r="C91" s="16" t="s">
+        <v>584</v>
+      </c>
+      <c r="D91" s="16" t="s">
         <v>585</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="16" t="s">
         <v>586</v>
-      </c>
-      <c r="E91" s="16" t="s">
-        <v>587</v>
       </c>
       <c r="F91" s="16" t="s">
         <v>58</v>
@@ -8574,34 +8571,34 @@
         <v>48</v>
       </c>
       <c r="N91" s="18" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="P91" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T91" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W91" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="X91" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y91" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="Z91" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="AA91" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="AB91" s="12" t="s">
         <v>684</v>
       </c>
-      <c r="X91" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Y91" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="Z91" s="23" t="s">
-        <v>684</v>
-      </c>
-      <c r="AA91" s="18" t="s">
-        <v>564</v>
-      </c>
-      <c r="AB91" s="12" t="s">
-        <v>685</v>
-      </c>
       <c r="AD91" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="92" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8612,13 +8609,13 @@
         <v>32</v>
       </c>
       <c r="C92" s="16" t="s">
+        <v>588</v>
+      </c>
+      <c r="D92" s="16" t="s">
         <v>589</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="E92" s="16" t="s">
         <v>590</v>
-      </c>
-      <c r="E92" s="16" t="s">
-        <v>591</v>
       </c>
       <c r="F92" s="16" t="s">
         <v>58</v>
@@ -8630,19 +8627,19 @@
         <v>467</v>
       </c>
       <c r="M92" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="N92" s="2" t="s">
         <v>698</v>
       </c>
-      <c r="N92" s="2" t="s">
-        <v>699</v>
-      </c>
       <c r="P92" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T92" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="V92" s="12" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="W92" s="16" t="s">
         <v>41</v>
@@ -8654,13 +8651,13 @@
         <v>92</v>
       </c>
       <c r="Z92" s="2" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="AA92" s="18" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="AD92" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="93" spans="1:30" ht="105" x14ac:dyDescent="0.25">
@@ -8671,13 +8668,13 @@
         <v>32</v>
       </c>
       <c r="C93" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="D93" s="16" t="s">
         <v>592</v>
       </c>
-      <c r="D93" s="16" t="s">
+      <c r="E93" s="16" t="s">
         <v>593</v>
-      </c>
-      <c r="E93" s="16" t="s">
-        <v>594</v>
       </c>
       <c r="F93" s="16" t="s">
         <v>58</v>
@@ -8692,34 +8689,34 @@
         <v>48</v>
       </c>
       <c r="N93" s="18" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="P93" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="T93" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="W93" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X93" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y93" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Z93" s="23" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA93" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB93" s="12" t="s">
+        <v>681</v>
+      </c>
+      <c r="AD93" s="2" t="s">
         <v>682</v>
-      </c>
-      <c r="AD93" s="2" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="94" spans="1:30" x14ac:dyDescent="0.25">
@@ -8730,13 +8727,13 @@
         <v>32</v>
       </c>
       <c r="C94" s="16" t="s">
+        <v>595</v>
+      </c>
+      <c r="D94" s="16" t="s">
         <v>596</v>
       </c>
-      <c r="D94" s="16" t="s">
+      <c r="E94" s="16" t="s">
         <v>597</v>
-      </c>
-      <c r="E94" s="16" t="s">
-        <v>598</v>
       </c>
       <c r="F94" s="16" t="s">
         <v>58</v>
@@ -8771,13 +8768,13 @@
         <v>32</v>
       </c>
       <c r="C95" s="16" t="s">
+        <v>598</v>
+      </c>
+      <c r="D95" s="16" t="s">
         <v>599</v>
       </c>
-      <c r="D95" s="16" t="s">
+      <c r="E95" s="16" t="s">
         <v>600</v>
-      </c>
-      <c r="E95" s="16" t="s">
-        <v>601</v>
       </c>
       <c r="F95" s="16" t="s">
         <v>58</v>
@@ -8812,13 +8809,13 @@
         <v>32</v>
       </c>
       <c r="C96" s="16" t="s">
+        <v>601</v>
+      </c>
+      <c r="D96" s="16" t="s">
         <v>602</v>
       </c>
-      <c r="D96" s="16" t="s">
+      <c r="E96" s="16" t="s">
         <v>603</v>
-      </c>
-      <c r="E96" s="16" t="s">
-        <v>604</v>
       </c>
       <c r="F96" s="16" t="s">
         <v>58</v>
@@ -8853,13 +8850,13 @@
         <v>32</v>
       </c>
       <c r="C97" s="16" t="s">
+        <v>604</v>
+      </c>
+      <c r="D97" s="16" t="s">
         <v>605</v>
       </c>
-      <c r="D97" s="16" t="s">
+      <c r="E97" s="16" t="s">
         <v>606</v>
-      </c>
-      <c r="E97" s="16" t="s">
-        <v>607</v>
       </c>
       <c r="F97" s="16" t="s">
         <v>58</v>
@@ -8894,13 +8891,13 @@
         <v>32</v>
       </c>
       <c r="C98" s="16" t="s">
+        <v>607</v>
+      </c>
+      <c r="D98" s="16" t="s">
         <v>608</v>
       </c>
-      <c r="D98" s="16" t="s">
+      <c r="E98" s="16" t="s">
         <v>609</v>
-      </c>
-      <c r="E98" s="16" t="s">
-        <v>610</v>
       </c>
       <c r="F98" s="16" t="s">
         <v>58</v>
@@ -8935,13 +8932,13 @@
         <v>32</v>
       </c>
       <c r="C99" s="16" t="s">
+        <v>610</v>
+      </c>
+      <c r="D99" s="16" t="s">
         <v>611</v>
       </c>
-      <c r="D99" s="16" t="s">
+      <c r="E99" s="16" t="s">
         <v>612</v>
-      </c>
-      <c r="E99" s="16" t="s">
-        <v>613</v>
       </c>
       <c r="F99" s="16" t="s">
         <v>58</v>
@@ -8976,13 +8973,13 @@
         <v>32</v>
       </c>
       <c r="C100" s="16" t="s">
+        <v>613</v>
+      </c>
+      <c r="D100" s="16" t="s">
         <v>614</v>
       </c>
-      <c r="D100" s="16" t="s">
+      <c r="E100" s="16" t="s">
         <v>615</v>
-      </c>
-      <c r="E100" s="16" t="s">
-        <v>616</v>
       </c>
       <c r="F100" s="16" t="s">
         <v>58</v>
@@ -9017,28 +9014,28 @@
         <v>32</v>
       </c>
       <c r="C101" s="16" t="s">
+        <v>616</v>
+      </c>
+      <c r="D101" s="16" t="s">
         <v>617</v>
       </c>
-      <c r="D101" s="16" t="s">
+      <c r="E101" s="16" t="s">
         <v>618</v>
-      </c>
-      <c r="E101" s="16" t="s">
-        <v>619</v>
       </c>
       <c r="F101" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J101" s="16" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="L101" s="17" t="s">
         <v>467</v>
       </c>
       <c r="M101" s="18" t="s">
+        <v>620</v>
+      </c>
+      <c r="N101" s="18" t="s">
         <v>621</v>
-      </c>
-      <c r="N101" s="18" t="s">
-        <v>622</v>
       </c>
       <c r="O101" s="16" t="s">
         <v>482</v>
@@ -9050,7 +9047,7 @@
         <v>470</v>
       </c>
       <c r="V101" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="W101" s="16" t="s">
         <v>41</v>
@@ -9065,10 +9062,10 @@
         <v>493</v>
       </c>
       <c r="AA101" s="18" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AC101" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="102" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -9079,19 +9076,19 @@
         <v>32</v>
       </c>
       <c r="C102" s="16" t="s">
+        <v>623</v>
+      </c>
+      <c r="D102" s="16" t="s">
         <v>624</v>
       </c>
-      <c r="D102" s="16" t="s">
+      <c r="E102" s="16" t="s">
         <v>625</v>
-      </c>
-      <c r="E102" s="16" t="s">
-        <v>626</v>
       </c>
       <c r="F102" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J102" s="16" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="L102" s="17" t="s">
         <v>467</v>
@@ -9113,10 +9110,10 @@
         <v>213</v>
       </c>
       <c r="AA102" s="18" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="AC102" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="103" spans="1:29" x14ac:dyDescent="0.25">
@@ -9127,19 +9124,19 @@
         <v>32</v>
       </c>
       <c r="C103" s="16" t="s">
+        <v>628</v>
+      </c>
+      <c r="D103" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="D103" s="16" t="s">
+      <c r="E103" s="16" t="s">
         <v>630</v>
-      </c>
-      <c r="E103" s="16" t="s">
-        <v>631</v>
       </c>
       <c r="F103" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J103" s="16" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="L103" s="17" t="s">
         <v>467</v>
@@ -9148,7 +9145,7 @@
         <v>48</v>
       </c>
       <c r="O103" s="16" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="W103" s="16" t="s">
         <v>213</v>
@@ -9171,19 +9168,19 @@
         <v>32</v>
       </c>
       <c r="C104" s="16" t="s">
+        <v>632</v>
+      </c>
+      <c r="D104" s="16" t="s">
         <v>633</v>
       </c>
-      <c r="D104" s="16" t="s">
-        <v>634</v>
-      </c>
       <c r="E104" s="16" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F104" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J104" s="16" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L104" s="17" t="s">
         <v>467</v>
@@ -9192,7 +9189,7 @@
         <v>48</v>
       </c>
       <c r="O104" s="16" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="W104" s="16" t="s">
         <v>213</v>
@@ -9215,19 +9212,19 @@
         <v>32</v>
       </c>
       <c r="C105" s="16" t="s">
+        <v>636</v>
+      </c>
+      <c r="D105" s="16" t="s">
         <v>637</v>
       </c>
-      <c r="D105" s="16" t="s">
-        <v>638</v>
-      </c>
       <c r="E105" s="16" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F105" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J105" s="16" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="L105" s="17" t="s">
         <v>467</v>
@@ -9236,7 +9233,7 @@
         <v>48</v>
       </c>
       <c r="O105" s="16" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="W105" s="16" t="s">
         <v>213</v>
@@ -9259,19 +9256,19 @@
         <v>32</v>
       </c>
       <c r="C106" s="16" t="s">
+        <v>639</v>
+      </c>
+      <c r="D106" s="16" t="s">
         <v>640</v>
       </c>
-      <c r="D106" s="16" t="s">
-        <v>641</v>
-      </c>
       <c r="E106" s="16" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F106" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J106" s="16" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="L106" s="17" t="s">
         <v>467</v>
@@ -9280,7 +9277,7 @@
         <v>48</v>
       </c>
       <c r="O106" s="16" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="W106" s="16" t="s">
         <v>213</v>
@@ -9303,19 +9300,19 @@
         <v>32</v>
       </c>
       <c r="C107" s="16" t="s">
+        <v>641</v>
+      </c>
+      <c r="D107" s="16" t="s">
         <v>642</v>
       </c>
-      <c r="D107" s="16" t="s">
-        <v>643</v>
-      </c>
       <c r="E107" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F107" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J107" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="M107" s="18" t="s">
         <v>48</v>
@@ -9341,19 +9338,19 @@
         <v>32</v>
       </c>
       <c r="C108" s="16" t="s">
+        <v>644</v>
+      </c>
+      <c r="D108" s="16" t="s">
         <v>645</v>
       </c>
-      <c r="D108" s="16" t="s">
-        <v>646</v>
-      </c>
       <c r="E108" s="16" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="F108" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J108" s="16" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="M108" s="18" t="s">
         <v>48</v>
@@ -9379,28 +9376,28 @@
         <v>32</v>
       </c>
       <c r="C109" s="16" t="s">
+        <v>647</v>
+      </c>
+      <c r="D109" s="16" t="s">
         <v>648</v>
       </c>
-      <c r="D109" s="16" t="s">
-        <v>649</v>
-      </c>
       <c r="E109" s="16" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F109" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J109" s="16" t="s">
+        <v>649</v>
+      </c>
+      <c r="M109" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="M109" s="18" t="s">
+      <c r="N109" s="18" t="s">
         <v>651</v>
       </c>
-      <c r="N109" s="18" t="s">
+      <c r="P109" s="16" t="s">
         <v>652</v>
-      </c>
-      <c r="P109" s="16" t="s">
-        <v>653</v>
       </c>
       <c r="T109" s="18" t="s">
         <v>91</v>
@@ -9415,16 +9412,16 @@
         <v>92</v>
       </c>
       <c r="Z109" s="19" t="s">
+        <v>653</v>
+      </c>
+      <c r="AA109" s="18" t="s">
         <v>654</v>
       </c>
-      <c r="AA109" s="18" t="s">
+      <c r="AB109" s="20" t="s">
         <v>655</v>
       </c>
-      <c r="AB109" s="20" t="s">
-        <v>656</v>
-      </c>
       <c r="AC109" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="110" spans="1:29" x14ac:dyDescent="0.25">
@@ -9435,19 +9432,19 @@
         <v>32</v>
       </c>
       <c r="C110" s="16" t="s">
+        <v>656</v>
+      </c>
+      <c r="D110" s="16" t="s">
         <v>657</v>
       </c>
-      <c r="D110" s="16" t="s">
-        <v>658</v>
-      </c>
       <c r="E110" s="16" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F110" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J110" s="16" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="M110" s="18" t="s">
         <v>48</v>
@@ -9465,7 +9462,7 @@
         <v>213</v>
       </c>
       <c r="AA110" s="17" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="111" spans="1:29" x14ac:dyDescent="0.25">
@@ -9476,22 +9473,22 @@
         <v>32</v>
       </c>
       <c r="C111" s="16" t="s">
+        <v>659</v>
+      </c>
+      <c r="D111" s="16" t="s">
         <v>660</v>
       </c>
-      <c r="D111" s="16" t="s">
-        <v>661</v>
-      </c>
       <c r="E111" s="16" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="F111" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J111" s="16" t="s">
+        <v>661</v>
+      </c>
+      <c r="K111" s="16" t="s">
         <v>662</v>
-      </c>
-      <c r="K111" s="16" t="s">
-        <v>663</v>
       </c>
       <c r="M111" s="18" t="s">
         <v>48</v>
@@ -9509,7 +9506,7 @@
         <v>213</v>
       </c>
       <c r="AA111" s="17" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="112" spans="1:29" x14ac:dyDescent="0.25">
@@ -9520,25 +9517,25 @@
         <v>32</v>
       </c>
       <c r="C112" s="16" t="s">
+        <v>663</v>
+      </c>
+      <c r="D112" s="16" t="s">
         <v>664</v>
       </c>
-      <c r="D112" s="16" t="s">
-        <v>665</v>
-      </c>
       <c r="E112" s="16" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="F112" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J112" s="16" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="M112" s="18" t="s">
         <v>48</v>
       </c>
       <c r="O112" s="16" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="W112" s="16" t="s">
         <v>213</v>
@@ -9553,7 +9550,7 @@
         <v>213</v>
       </c>
       <c r="AA112" s="17" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="113" spans="1:27" x14ac:dyDescent="0.25">
@@ -9564,19 +9561,19 @@
         <v>32</v>
       </c>
       <c r="C113" s="16" t="s">
+        <v>666</v>
+      </c>
+      <c r="D113" s="16" t="s">
         <v>667</v>
       </c>
-      <c r="D113" s="16" t="s">
-        <v>668</v>
-      </c>
       <c r="E113" s="16" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F113" s="16" t="s">
         <v>58</v>
       </c>
       <c r="J113" s="16" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="M113" s="18" t="s">
         <v>48</v>
@@ -9594,7 +9591,7 @@
         <v>213</v>
       </c>
       <c r="AA113" s="17" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix for CVD ever
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-BCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9832A0F6-2A33-4765-9E49-BED7F11A0A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F814562-DDD1-4946-BB7F-4DCBB9DDBDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="789">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1747" uniqueCount="791">
   <si>
     <t>index</t>
   </si>
@@ -2908,12 +2908,6 @@
 Health problems since last interview/2016: Heart problems;
 Health problems since last interview/2016: Stroke;
 Health problems since last interview/2016: None of these</t>
-  </si>
-  <si>
-    <t>case_when(
-b11khlpb06 == 1 | b11khlpb08 == 1 | b11khlpb09 == 1 ~ 1L; 
-b11khlpb10 == 1 ~ 2L ;
-ELSE ~ NA_integer_)</t>
   </si>
   <si>
     <t xml:space="preserve">(-9) Refused (-8) Don't know (-3) Not asked at case fieldwork stage (-2) Not asked due to scripting/routing error (-1) Not applicable (0) Not mentioned (1) Mentioned </t>
@@ -3206,6 +3200,19 @@
 Coding for study category 6? (not coded).
 Also a variable BD10ANVQ, but everyone with info for BD10ANVQ has BD10HACHQ. -&gt; Many people have NVQ = 0.
 </t>
+  </si>
+  <si>
+    <t>The study-specific variables ask about types of health problems since last interview/2016.
+The study-specific variables are in select-all-that-apply format, so only Presumed no can be coded.  Participants were presumed not to have CVD if they did not select high blood pressure, heart problems, or stroke.</t>
+  </si>
+  <si>
+    <t>case_when(
+b11khlpb06 == 1 | b11khlpb08 == 1 | b11khlpb09 == 1 ~ 1L; 
+b11khlpb10 %in% c(0,1) ~ 2L ;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>Updated to presume no for anyone that didn't select high blood pressure, heart problems, or stroke. Previous rule was much more conservative.</t>
   </si>
 </sst>
 </file>
@@ -3313,7 +3320,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3392,6 +3399,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3759,7 +3772,7 @@
     <col min="28" max="28" width="42.28515625" style="18" customWidth="1"/>
     <col min="29" max="29" width="41.7109375" style="18" customWidth="1"/>
     <col min="30" max="30" width="32.85546875" style="18" customWidth="1"/>
-    <col min="31" max="31" width="21" style="16" customWidth="1"/>
+    <col min="31" max="31" width="26.42578125" style="16" customWidth="1"/>
     <col min="32" max="32" width="16.140625" style="16" customWidth="1"/>
     <col min="33" max="33" width="14.28515625" style="16" customWidth="1"/>
     <col min="34" max="34" width="9" style="16" customWidth="1"/>
@@ -3774,7 +3787,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -3987,7 +4000,7 @@
         <v>50</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -4222,10 +4235,10 @@
         <v>99</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="S9" s="16" t="s">
         <v>58</v>
@@ -4255,7 +4268,7 @@
         <v>703</v>
       </c>
       <c r="AC9" s="11" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="AD9" s="24" t="s">
         <v>704</v>
@@ -4311,7 +4324,7 @@
         <v>79</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="AC10" s="12" t="s">
         <v>705</v>
@@ -5977,10 +5990,10 @@
         <v>297</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="O45" s="23" t="s">
         <v>298</v>
@@ -6005,7 +6018,7 @@
         <v>92</v>
       </c>
       <c r="Z45" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="AA45" s="18" t="s">
         <v>299</v>
@@ -6014,7 +6027,7 @@
         <v>300</v>
       </c>
       <c r="AC45" s="2" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="AD45" s="19" t="s">
         <v>674</v>
@@ -6192,7 +6205,7 @@
         <v>79</v>
       </c>
       <c r="Z48" s="2" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="49" spans="1:30" ht="75" x14ac:dyDescent="0.25">
@@ -6478,13 +6491,13 @@
         <v>92</v>
       </c>
       <c r="Z53" s="2" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="AA53" s="18" t="s">
         <v>356</v>
       </c>
       <c r="AC53" s="2" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="54" spans="1:30" ht="150" x14ac:dyDescent="0.25">
@@ -7028,7 +7041,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="65" spans="1:30" ht="300" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" ht="300" x14ac:dyDescent="0.25">
       <c r="A65" s="16">
         <v>64</v>
       </c>
@@ -7057,7 +7070,7 @@
         <v>107</v>
       </c>
       <c r="M65" s="18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="N65" s="18" t="s">
         <v>429</v>
@@ -7087,7 +7100,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="66" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" ht="75" x14ac:dyDescent="0.25">
       <c r="A66" s="16">
         <v>65</v>
       </c>
@@ -7143,7 +7156,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="67" spans="1:30" ht="150" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" ht="150" x14ac:dyDescent="0.25">
       <c r="A67" s="16">
         <v>66</v>
       </c>
@@ -7193,7 +7206,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="68" spans="1:30" ht="150" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" ht="150" x14ac:dyDescent="0.25">
       <c r="A68" s="16">
         <v>67</v>
       </c>
@@ -7246,7 +7259,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="69" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" ht="105" x14ac:dyDescent="0.25">
       <c r="A69" s="16">
         <v>68</v>
       </c>
@@ -7289,8 +7302,8 @@
       <c r="T69" s="21" t="s">
         <v>470</v>
       </c>
-      <c r="V69" s="12" t="s">
-        <v>779</v>
+      <c r="V69" s="27" t="s">
+        <v>788</v>
       </c>
       <c r="W69" s="16" t="s">
         <v>41</v>
@@ -7301,8 +7314,8 @@
       <c r="Y69" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="Z69" s="2" t="s">
-        <v>748</v>
+      <c r="Z69" s="28" t="s">
+        <v>789</v>
       </c>
       <c r="AA69" s="18" t="s">
         <v>471</v>
@@ -7313,8 +7326,11 @@
       <c r="AC69" s="12" t="s">
         <v>745</v>
       </c>
-    </row>
-    <row r="70" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+      <c r="AE69" s="27" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="70" spans="1:31" ht="75" x14ac:dyDescent="0.25">
       <c r="A70" s="16">
         <v>69</v>
       </c>
@@ -7343,10 +7359,10 @@
         <v>467</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="O70" s="23" t="s">
         <v>468</v>
@@ -7356,10 +7372,10 @@
       <c r="R70" s="23"/>
       <c r="S70" s="23"/>
       <c r="T70" s="2" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="V70" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W70" s="23" t="s">
         <v>41</v>
@@ -7371,16 +7387,16 @@
         <v>92</v>
       </c>
       <c r="Z70" s="2" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="AB70" s="18" t="s">
         <v>672</v>
       </c>
       <c r="AC70" s="2" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="71" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="71" spans="1:31" ht="75" x14ac:dyDescent="0.25">
       <c r="A71" s="16">
         <v>70</v>
       </c>
@@ -7409,10 +7425,10 @@
         <v>467</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="O71" s="23" t="s">
         <v>482</v>
@@ -7422,10 +7438,10 @@
       <c r="R71" s="23"/>
       <c r="S71" s="23"/>
       <c r="T71" s="2" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="V71" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W71" s="23" t="s">
         <v>41</v>
@@ -7437,13 +7453,13 @@
         <v>92</v>
       </c>
       <c r="Z71" s="2" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="AC71" s="2" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="72" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="72" spans="1:31" ht="75" x14ac:dyDescent="0.25">
       <c r="A72" s="16">
         <v>71</v>
       </c>
@@ -7472,10 +7488,10 @@
         <v>467</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="O72" s="23" t="s">
         <v>482</v>
@@ -7485,10 +7501,10 @@
       <c r="R72" s="23"/>
       <c r="S72" s="23"/>
       <c r="T72" s="2" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="V72" s="12" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="W72" s="23" t="s">
         <v>41</v>
@@ -7500,13 +7516,13 @@
         <v>92</v>
       </c>
       <c r="Z72" s="2" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="AC72" s="2" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="73" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="73" spans="1:31" ht="105" x14ac:dyDescent="0.25">
       <c r="A73" s="16">
         <v>72</v>
       </c>
@@ -7550,7 +7566,7 @@
         <v>470</v>
       </c>
       <c r="V73" s="12" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>41</v>
@@ -7562,16 +7578,16 @@
         <v>79</v>
       </c>
       <c r="Z73" s="2" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="AA73" s="18" t="s">
         <v>494</v>
       </c>
       <c r="AC73" s="2" t="s">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="74" spans="1:30" x14ac:dyDescent="0.25">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="74" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A74" s="16">
         <v>73</v>
       </c>
@@ -7618,7 +7634,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="75" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A75" s="16">
         <v>74</v>
       </c>
@@ -7662,10 +7678,10 @@
         <v>213</v>
       </c>
       <c r="AC75" s="18" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="76" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="76" spans="1:31" ht="105" x14ac:dyDescent="0.25">
       <c r="A76" s="16">
         <v>75</v>
       </c>
@@ -7712,7 +7728,7 @@
         <v>470</v>
       </c>
       <c r="V76" s="12" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="W76" s="16" t="s">
         <v>41</v>
@@ -7724,16 +7740,16 @@
         <v>79</v>
       </c>
       <c r="Z76" s="2" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="AA76" s="18" t="s">
         <v>511</v>
       </c>
       <c r="AC76" s="2" t="s">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="77" spans="1:30" x14ac:dyDescent="0.25">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="77" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A77" s="16">
         <v>76</v>
       </c>
@@ -7777,10 +7793,10 @@
         <v>213</v>
       </c>
       <c r="AC77" s="18" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="78" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="78" spans="1:31" ht="90" x14ac:dyDescent="0.25">
       <c r="A78" s="16">
         <v>77</v>
       </c>
@@ -7809,17 +7825,17 @@
         <v>467</v>
       </c>
       <c r="M78" s="2" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="O78" s="16" t="s">
         <v>521</v>
       </c>
       <c r="T78" s="2"/>
       <c r="V78" s="12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="W78" s="23" t="s">
         <v>41</v>
@@ -7831,13 +7847,13 @@
         <v>79</v>
       </c>
       <c r="Z78" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="AB78" s="11" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="79" spans="1:30" ht="135" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" ht="135" x14ac:dyDescent="0.25">
       <c r="A79" s="16">
         <v>78</v>
       </c>
@@ -7893,7 +7909,7 @@
         <v>79</v>
       </c>
       <c r="Z79" s="2" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AA79" s="18" t="s">
         <v>529</v>
@@ -7902,10 +7918,10 @@
         <v>472</v>
       </c>
       <c r="AC79" s="2" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="80" spans="1:30" x14ac:dyDescent="0.25">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="80" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A80" s="16">
         <v>79</v>
       </c>
@@ -7993,7 +8009,7 @@
         <v>470</v>
       </c>
       <c r="V81" s="12" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="W81" s="16" t="s">
         <v>41</v>
@@ -8108,7 +8124,7 @@
         <v>552</v>
       </c>
       <c r="V83" s="12" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="W83" s="16" t="s">
         <v>41</v>
@@ -8120,7 +8136,7 @@
         <v>92</v>
       </c>
       <c r="Z83" s="2" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AA83" s="18" t="s">
         <v>553</v>
@@ -8639,7 +8655,7 @@
         <v>552</v>
       </c>
       <c r="V92" s="12" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="W92" s="16" t="s">
         <v>41</v>
@@ -8651,7 +8667,7 @@
         <v>92</v>
       </c>
       <c r="Z92" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="AA92" s="18" t="s">
         <v>553</v>

</xml_diff>